<commit_message>
Apply reviewed machine-zone table and add water station zone
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCF3bZGqLBzEM7DVQ348XJ
</commit_message>
<xml_diff>
--- a/production-downtime-app/Table_zones_laminoir.xlsx
+++ b/production-downtime-app/Table_zones_laminoir.xlsx
@@ -63,9 +63,7 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -468,7 +466,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -483,7 +481,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -498,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -513,7 +511,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -528,7 +526,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -543,7 +541,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -558,7 +556,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -573,7 +571,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -588,7 +586,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -603,7 +601,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -618,7 +616,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -633,7 +631,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -648,7 +646,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -663,7 +661,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -678,7 +676,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -693,7 +691,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -708,7 +706,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -723,7 +721,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -738,7 +736,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -753,7 +751,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -768,7 +766,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -783,7 +781,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -798,7 +796,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -813,7 +811,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -828,7 +826,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -843,7 +841,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -858,7 +856,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -873,7 +871,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -888,7 +886,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -903,7 +901,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -918,7 +916,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -933,7 +931,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -948,7 +946,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -963,7 +961,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -978,7 +976,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -993,7 +991,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1006,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1021,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Hors schéma</t>
+          <t>Station eau</t>
         </is>
       </c>
     </row>
@@ -2343,7 +2341,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Train</t>
+          <t>Ligne petit diamètre</t>
         </is>
       </c>
     </row>
@@ -2358,7 +2356,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Train</t>
+          <t>Ligne petit diamètre</t>
         </is>
       </c>
     </row>
@@ -2778,7 +2776,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Refroidissoir jusque VR9</t>
+          <t>Ligne gros diamètre</t>
         </is>
       </c>
     </row>
@@ -2793,7 +2791,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Refroidissoir jusque VR9</t>
+          <t>Ligne gros diamètre</t>
         </is>
       </c>
     </row>
@@ -2808,7 +2806,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Refroidissoir jusque VR9</t>
+          <t>Ligne gros diamètre</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2821,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Refroidissoir jusque VR9</t>
+          <t>Ligne gros diamètre</t>
         </is>
       </c>
     </row>
@@ -2838,7 +2836,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Refroidissoir jusque VR9</t>
+          <t>Ligne gros diamètre</t>
         </is>
       </c>
     </row>
@@ -2853,7 +2851,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Refroidissoir jusque VR9</t>
+          <t>Ligne gros diamètre</t>
         </is>
       </c>
     </row>
@@ -2868,7 +2866,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Refroidissoir jusque VR9</t>
+          <t>Ligne gros diamètre</t>
         </is>
       </c>
     </row>
@@ -3595,8 +3593,8 @@
   </sheetData>
   <autoFilter ref="A1:C210"/>
   <dataValidations count="1">
-    <dataValidation sqref="C2:C210" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Zone inconnue" error="Choisissez une zone de la liste." type="list">
-      <formula1>='Liste zones'!$A$2:$A$10</formula1>
+    <dataValidation sqref="C2:C210" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>='Liste zones'!$A$2:$A$11</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3609,7 +3607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3681,6 +3679,13 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Station eau</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Hors schéma</t>
         </is>
       </c>

</xml_diff>